<commit_message>
feat: agregar plantillas de evaluación para Amazon, Costco y Nike
Agrega hojas de cálculo de prueba para las evaluaciones de Amazon,
Costco y Nike, y actualiza la plantilla existente de Nvidia.
</commit_message>
<xml_diff>
--- a/docs/plantillas-de-valorizacion/evaluaciones/Nvidia.xlsx
+++ b/docs/plantillas-de-valorizacion/evaluaciones/Nvidia.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10412"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247CFBFD-DD87-EA48-833E-88621FBA5B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E97B6E1-2753-3F4C-80A9-6791C5EB0407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40" yWindow="700" windowWidth="30160" windowHeight="18900" tabRatio="636" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="25620" yWindow="640" windowWidth="25560" windowHeight="20920" tabRatio="636" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucciones" sheetId="13" r:id="rId1"/>

</xml_diff>